<commit_message>
chore(results): update result outputs
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -582,8 +582,8 @@
     <col width="16.8" customWidth="1" min="1" max="1"/>
     <col width="9.6" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="25.2" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="26.4" customWidth="1" min="4" max="4"/>
+    <col width="22.8" customWidth="1" min="5" max="5"/>
     <col width="34.8" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="15.6" customWidth="1" min="8" max="8"/>
@@ -642,16 +642,16 @@
         <v>1364</v>
       </c>
       <c r="C2" t="n">
-        <v>1.637028026319269</v>
+        <v>1.668284021994126</v>
       </c>
       <c r="D2" t="n">
-        <v>0.07413839991204441</v>
+        <v>0.07034079999993992</v>
       </c>
       <c r="E2" t="n">
-        <v>19.76585069997236</v>
+        <v>20.03505740000037</v>
       </c>
       <c r="F2" t="n">
-        <v>2.700202219999627</v>
+        <v>2.70657735309327</v>
       </c>
       <c r="G2" t="n">
         <v>377</v>
@@ -673,16 +673,16 @@
         <v>1741</v>
       </c>
       <c r="C3" t="n">
-        <v>9.27714340247271</v>
+        <v>0.4458798143021125</v>
       </c>
       <c r="D3" t="n">
-        <v>0.02228619996458292</v>
+        <v>0.01555959999950574</v>
       </c>
       <c r="E3" t="n">
-        <v>134.5009773001075</v>
+        <v>4.553129700000682</v>
       </c>
       <c r="F3" t="n">
-        <v>15.58795169480885</v>
+        <v>0.6595615547299756</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -729,7 +729,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1399</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="3">
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>899</v>
+        <v>902</v>
       </c>
     </row>
     <row r="4">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>142.4537622056289</v>
+        <v>142.6111430212522</v>
       </c>
     </row>
     <row r="5">
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>288.0614479167753</v>
+        <v>288.0970360969133</v>
       </c>
     </row>
     <row r="8">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0.005294163506840346</v>
+        <v>0.005298414518979526</v>
       </c>
     </row>
     <row r="9">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>79.01206203331419</v>
+        <v>79.23721998851235</v>
       </c>
     </row>
     <row r="10">
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>188.1529141318901</v>
+        <v>188.2191565873644</v>
       </c>
     </row>
     <row r="13">
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>0.001385859227250776</v>
+        <v>0.001388967351654756</v>
       </c>
     </row>
     <row r="14">
@@ -849,7 +849,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>96.4744399770247</v>
+        <v>96.54106835152211</v>
       </c>
     </row>
     <row r="15">
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>185.8083788599272</v>
+        <v>185.8218844072151</v>
       </c>
     </row>
     <row r="18">
@@ -899,7 +899,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>20.98506605399196</v>
+        <v>21.02125215393452</v>
       </c>
     </row>
     <row r="20">
@@ -929,7 +929,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>47.63407337631442</v>
+        <v>47.64333682427053</v>
       </c>
     </row>
     <row r="23">
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>255851.5502584722</v>
+        <v>255847.8047099368</v>
       </c>
     </row>
     <row r="25">
@@ -979,7 +979,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>821221.1295896077</v>
+        <v>821221.9387553548</v>
       </c>
     </row>
     <row r="28">
@@ -999,7 +999,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.2260437532558736</v>
+        <v>0.205216401571435</v>
       </c>
     </row>
     <row r="30">
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0.002478100126609206</v>
+        <v>0.002454099999340542</v>
       </c>
     </row>
     <row r="31">
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>5.287629700032994</v>
+        <v>4.232367100000374</v>
       </c>
     </row>
     <row r="32">
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.4188840566508125</v>
+        <v>0.3643761242375684</v>
       </c>
     </row>
     <row r="33">
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0.04494465228524452</v>
+        <v>0.04612594623058673</v>
       </c>
     </row>
     <row r="34">
@@ -1049,7 +1049,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.001580100040882826</v>
+        <v>0.001757199999701697</v>
       </c>
     </row>
     <row r="35">
@@ -1059,7 +1059,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.6443039998412132</v>
+        <v>0.6979713999999149</v>
       </c>
     </row>
     <row r="36">
@@ -1069,7 +1069,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.07048896526610463</v>
+        <v>0.07278276081733959</v>
       </c>
     </row>
     <row r="37">
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.2678180044935485</v>
+        <v>0.248295962633462</v>
       </c>
     </row>
     <row r="38">
@@ -1089,7 +1089,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.004402599995955825</v>
+        <v>0.0042462000001251</v>
       </c>
     </row>
     <row r="39">
@@ -1099,7 +1099,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>5.54835609998554</v>
+        <v>4.508044700000028</v>
       </c>
     </row>
     <row r="40">
@@ -1109,7 +1109,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.456738180170365</v>
+        <v>0.4063733386373479</v>
       </c>
     </row>
     <row r="41">
@@ -1119,7 +1119,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.001882778311790567</v>
+        <v>0.001709343056200151</v>
       </c>
     </row>
     <row r="42">
@@ -1129,7 +1129,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.001105932459407002</v>
+        <v>0.001136827244657884</v>
       </c>
     </row>
     <row r="43">
@@ -1139,7 +1139,7 @@
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>0.193865156358877</v>
+        <v>0.1736163444433252</v>
       </c>
     </row>
     <row r="44">
@@ -1149,7 +1149,7 @@
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>0.005792744260493589</v>
+        <v>0.005332059666288169</v>
       </c>
     </row>
     <row r="45">
@@ -1159,7 +1159,7 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>1.807223083055872</v>
+        <v>1.46985218304692</v>
       </c>
     </row>
     <row r="46">
@@ -1169,7 +1169,7 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>0.200795580733024</v>
+        <v>0.1688421987087319</v>
       </c>
     </row>
     <row r="47">
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>0.03345828574217863</v>
+        <v>0.8782542614431649</v>
       </c>
     </row>
     <row r="48">
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>0.001300110888397616</v>
+        <v>0.003705109211835135</v>
       </c>
     </row>
     <row r="49">
@@ -1199,7 +1199,7 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>0.5393655632089471</v>
+        <v>14.64854829349409</v>
       </c>
     </row>
     <row r="50">
@@ -1209,7 +1209,7 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>0.04975169088978405</v>
+        <v>1.27082854759706</v>
       </c>
     </row>
     <row r="51">

</xml_diff>